<commit_message>
added "ВНА" column in excel export of parameters
</commit_message>
<xml_diff>
--- a/results/поступенчатый_расчет_ступеней.xlsx
+++ b/results/поступенчатый_расчет_ступеней.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -430,13 +430,14 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -447,60 +448,65 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Название (из комментария)</t>
+          <t>Название</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>ВНА</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Ступень 1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ступень 2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Ступень 3</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Ступень 4</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ступень 5</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Ступень 6</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Ступень 7</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Ступень 8</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Ступень 9</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Ступень 10</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Ступень 11</t>
         </is>
@@ -530,6 +536,7 @@
       <c r="K2" s="1" t="inlineStr"/>
       <c r="L2" s="1" t="inlineStr"/>
       <c r="M2" s="1" t="inlineStr"/>
+      <c r="N2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -555,6 +562,7 @@
       <c r="K3" s="1" t="inlineStr"/>
       <c r="L3" s="1" t="inlineStr"/>
       <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -580,6 +588,7 @@
       <c r="K4" s="1" t="inlineStr"/>
       <c r="L4" s="1" t="inlineStr"/>
       <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -605,6 +614,7 @@
       <c r="K5" s="1" t="inlineStr"/>
       <c r="L5" s="1" t="inlineStr"/>
       <c r="M5" s="1" t="inlineStr"/>
+      <c r="N5" s="1" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -630,6 +640,7 @@
       <c r="K6" s="1" t="inlineStr"/>
       <c r="L6" s="1" t="inlineStr"/>
       <c r="M6" s="1" t="inlineStr"/>
+      <c r="N6" s="1" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -642,37 +653,38 @@
           <t>Показатель адиабаты по длине компрессора перед РК</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="1" t="inlineStr"/>
+      <c r="D7" s="2" t="n">
         <v>1.399944336209296</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="E7" s="2" t="n">
         <v>1.397730417935234</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>1.395170974280756</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>1.392955452904169</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>1.389895378447053</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="I7" s="2" t="n">
         <v>1.38614429252978</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="J7" s="2" t="n">
         <v>1.382383207491211</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>1.377411819293562</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="L7" s="2" t="n">
         <v>1.373497531831458</v>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="M7" s="2" t="n">
         <v>1.369326438894018</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="N7" s="2" t="n">
         <v>1.364941218981699</v>
       </c>
     </row>
@@ -687,37 +699,38 @@
           <t>Коэффициент расхода на входе в ступень</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="1" t="inlineStr"/>
+      <c r="D8" s="2" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="E8" s="2" t="n">
         <v>0.54</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>0.52</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>0.48</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="I8" s="2" t="n">
         <v>0.46</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="J8" s="2" t="n">
         <v>0.44</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="K8" s="2" t="n">
         <v>0.42</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="L8" s="2" t="n">
         <v>0.4</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="M8" s="2" t="n">
         <v>0.38</v>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>0.36</v>
       </c>
     </row>
@@ -732,37 +745,38 @@
           <t>Коэффициент расхода на выходе из ступени</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="2" t="n">
         <v>0.54</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="E9" s="2" t="n">
         <v>0.52</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>0.48</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>0.46</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="I9" s="2" t="n">
         <v>0.44</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="J9" s="2" t="n">
         <v>0.42</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>0.4</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>0.38</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="M9" s="2" t="n">
         <v>0.36</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>0.34</v>
       </c>
     </row>
@@ -777,37 +791,38 @@
           <t>Полное давление перед ступенью</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="2" t="n">
         <v>100454.5780155997</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="E10" s="2" t="n">
         <v>275692.1766287496</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>450929.7752418994</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>626167.3738550491</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>801404.972468199</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="I10" s="2" t="n">
         <v>976642.5710813488</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="J10" s="2" t="n">
         <v>1151880.169694499</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="K10" s="2" t="n">
         <v>1327117.768307649</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="L10" s="2" t="n">
         <v>1502355.366920798</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="M10" s="2" t="n">
         <v>1677592.965533948</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>1852830.564147098</v>
       </c>
     </row>
@@ -822,37 +837,38 @@
           <t>Полная температура перед ступенью</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="2" t="n">
         <v>288</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="E11" s="2" t="n">
         <v>327.5017025887266</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>367.0034051774532</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>406.5051077661798</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>446.0068103549064</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="I11" s="2" t="n">
         <v>485.508512943633</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="J11" s="2" t="n">
         <v>525.0102155323597</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="K11" s="2" t="n">
         <v>564.5119181210862</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="L11" s="2" t="n">
         <v>604.0136207098128</v>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="M11" s="2" t="n">
         <v>643.5153232985394</v>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>683.0170258872661</v>
       </c>
     </row>
@@ -867,37 +883,38 @@
           <t>Относительный диаметр втулки на входе в ступень</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="2" t="n">
         <v>0.43</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="E12" s="2" t="n">
         <v>0.4798027938858659</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="F12" s="2" t="n">
         <v>0.5296055877717317</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>0.5794083816575977</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>0.6292111755434635</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="I12" s="2" t="n">
         <v>0.6790139694293295</v>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="J12" s="2" t="n">
         <v>0.7288167633151953</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="K12" s="2" t="n">
         <v>0.7786195572010612</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="L12" s="2" t="n">
         <v>0.8284223510869271</v>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="M12" s="2" t="n">
         <v>0.8782251449727929</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="N12" s="2" t="n">
         <v>0.9280279388586589</v>
       </c>
     </row>
@@ -912,9 +929,7 @@
           <t>Окружная скорость концов рабочих лопаток ступени</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
-        <v>320.1197013603089</v>
-      </c>
+      <c r="C13" s="1" t="inlineStr"/>
       <c r="D13" s="2" t="n">
         <v>320.1197013603089</v>
       </c>
@@ -945,6 +960,9 @@
       <c r="M13" s="2" t="n">
         <v>320.1197013603089</v>
       </c>
+      <c r="N13" s="2" t="n">
+        <v>320.1197013603089</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
@@ -957,37 +975,38 @@
           <t>Теоретический напор i-й ступени</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="2" t="n">
         <v>25854.19789646718</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="E14" s="2" t="n">
         <v>27331.55639301205</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="F14" s="2" t="n">
         <v>28757.69684116139</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>30128.18965931852</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>31434.22303533384</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="I14" s="2" t="n">
         <v>32665.1866306543</v>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="J14" s="2" t="n">
         <v>33804.74258016107</v>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="K14" s="2" t="n">
         <v>34833.47648090584</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="L14" s="2" t="n">
         <v>35728.22725626807</v>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="M14" s="2" t="n">
         <v>36462.08715595525</v>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>37004.40175600272</v>
       </c>
     </row>
@@ -1002,37 +1021,38 @@
           <t>Действительная работа сжатия i-й ступени</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="2" t="n">
         <v>25595.65591750251</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="E15" s="2" t="n">
         <v>26784.92526515181</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="F15" s="2" t="n">
         <v>27894.96593592654</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>28923.06207294577</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>29862.51188356715</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="I15" s="2" t="n">
         <v>30705.27543281504</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="J15" s="2" t="n">
         <v>31776.45802535141</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K15" s="2" t="n">
         <v>32743.46789205149</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>33584.53362089198</v>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="M15" s="2" t="n">
         <v>34274.36192659794</v>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>34784.13765064256</v>
       </c>
     </row>
@@ -1047,37 +1067,38 @@
           <t>Адиабатическая работа сжатия i-й ступени</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="2" t="n">
         <v>22295.90245529727</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="E16" s="2" t="n">
         <v>23523.8609963345</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="F16" s="2" t="n">
         <v>24641.8293462309</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>25637.21001079051</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>26494.61026037706</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="I16" s="2" t="n">
         <v>27198.36428680719</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="J16" s="2" t="n">
         <v>28027.72920951312</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>28679.12596132233</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>29126.47125574586</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="M16" s="2" t="n">
         <v>29343.0094878997</v>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="N16" s="2" t="n">
         <v>29302.19111187581</v>
       </c>
     </row>
@@ -1092,37 +1113,38 @@
           <t>Повышение полной температуры в ступени</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="2" t="n">
         <v>25.44299792992297</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="E17" s="2" t="n">
         <v>26.51972798529882</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="F17" s="2" t="n">
         <v>27.49138860665853</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>28.38988267523888</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>29.14778438952522</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="I17" s="2" t="n">
         <v>29.76236322732219</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="J17" s="2" t="n">
         <v>30.58363382072301</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>31.21688767539521</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="L17" s="2" t="n">
         <v>31.77696465013327</v>
       </c>
-      <c r="L17" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>32.16518247860331</v>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="N17" s="2" t="n">
         <v>32.35962250431123</v>
       </c>
     </row>
@@ -1137,37 +1159,38 @@
           <t>Полная температура на выходе из ступени</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="2" t="n">
         <v>313.442997929923</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="E18" s="2" t="n">
         <v>354.0214305740254</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="F18" s="2" t="n">
         <v>394.4947937841117</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>434.8949904414187</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>475.1545947444316</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="I18" s="2" t="n">
         <v>515.2708761709553</v>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="J18" s="2" t="n">
         <v>555.5938493530826</v>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="K18" s="2" t="n">
         <v>595.7288057964814</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="L18" s="2" t="n">
         <v>635.7905853599461</v>
       </c>
-      <c r="L18" s="2" t="n">
+      <c r="M18" s="2" t="n">
         <v>675.6805057771428</v>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="N18" s="2" t="n">
         <v>715.3766483915773</v>
       </c>
     </row>
@@ -1182,37 +1205,38 @@
           <t>Полная температура на входе в следующую ступень</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="1" t="inlineStr"/>
+      <c r="D19" s="2" t="n">
         <v>313.442997929923</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="E19" s="2" t="n">
         <v>354.0214305740254</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="F19" s="2" t="n">
         <v>394.4947937841117</v>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>434.8949904414187</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>475.1545947444316</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="I19" s="2" t="n">
         <v>515.2708761709553</v>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="J19" s="2" t="n">
         <v>555.5938493530826</v>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="K19" s="2" t="n">
         <v>595.7288057964814</v>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="L19" s="2" t="n">
         <v>635.7905853599461</v>
       </c>
-      <c r="L19" s="2" t="n">
+      <c r="M19" s="2" t="n">
         <v>675.6805057771428</v>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="N19" s="2" t="n">
         <v>715.3766483915773</v>
       </c>
     </row>
@@ -1227,37 +1251,38 @@
           <t>Степень повышения полного давления в ступени</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="1" t="inlineStr"/>
+      <c r="D20" s="2" t="n">
         <v>1.296289753371198</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="E20" s="2" t="n">
         <v>1.273077659708594</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="F20" s="2" t="n">
         <v>1.253849641297374</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>1.237281701016347</v>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>1.22253229938774</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="I20" s="2" t="n">
         <v>1.209023758265309</v>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="J20" s="2" t="n">
         <v>1.198579725967046</v>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="K20" s="2" t="n">
         <v>1.188416178809493</v>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="L20" s="2" t="n">
         <v>1.178297216252501</v>
       </c>
-      <c r="L20" s="2" t="n">
+      <c r="M20" s="2" t="n">
         <v>1.168073869324779</v>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="N20" s="2" t="n">
         <v>1.157625977031957</v>
       </c>
     </row>
@@ -1272,37 +1297,38 @@
           <t>Полное давление на выходе из ступени</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="1" t="inlineStr"/>
+      <c r="D21" s="2" t="n">
         <v>130218.2401608496</v>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="E21" s="2" t="n">
         <v>350977.5510224969</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="F21" s="2" t="n">
         <v>565398.1369373611</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>774745.4334443138</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>979743.4637323158</v>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="I21" s="2" t="n">
         <v>1180784.071770667</v>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="J21" s="2" t="n">
         <v>1380620.218139306</v>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="K21" s="2" t="n">
         <v>1577168.227042358</v>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="L21" s="2" t="n">
         <v>1770221.14666478</v>
       </c>
-      <c r="L21" s="2" t="n">
+      <c r="M21" s="2" t="n">
         <v>1959552.50640327</v>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="N21" s="2" t="n">
         <v>2144884.792095456</v>
       </c>
     </row>
@@ -1317,37 +1343,38 @@
           <t>Полное давление перед следующей ступенью</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C22" s="1" t="inlineStr"/>
+      <c r="D22" s="2" t="n">
         <v>130218.2401608496</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="E22" s="2" t="n">
         <v>350977.5510224969</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="F22" s="2" t="n">
         <v>565398.1369373611</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>774745.4334443138</v>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="H22" s="2" t="n">
         <v>979743.4637323158</v>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="I22" s="2" t="n">
         <v>1180784.071770667</v>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="J22" s="2" t="n">
         <v>1380620.218139306</v>
       </c>
-      <c r="J22" s="2" t="n">
+      <c r="K22" s="2" t="n">
         <v>1577168.227042358</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="L22" s="2" t="n">
         <v>1770221.14666478</v>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="M22" s="2" t="n">
         <v>1959552.50640327</v>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="N22" s="2" t="n">
         <v>2144884.792095456</v>
       </c>
     </row>
@@ -1362,37 +1389,38 @@
           <t>Критическая скорость потока на входе в ступень</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C23" s="1" t="inlineStr"/>
+      <c r="D23" s="2" t="n">
         <v>310.7487734256569</v>
       </c>
-      <c r="D23" s="2" t="n">
+      <c r="E23" s="2" t="n">
         <v>331.2658695389746</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="F23" s="2" t="n">
         <v>350.5410496913398</v>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>368.8015096578053</v>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>386.12750213934</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="I23" s="2" t="n">
         <v>402.6360656708928</v>
       </c>
-      <c r="I23" s="2" t="n">
+      <c r="J23" s="2" t="n">
         <v>418.456840685445</v>
       </c>
-      <c r="J23" s="2" t="n">
+      <c r="K23" s="2" t="n">
         <v>433.5853814040989</v>
       </c>
-      <c r="K23" s="2" t="n">
+      <c r="L23" s="2" t="n">
         <v>448.2303868459118</v>
       </c>
-      <c r="L23" s="2" t="n">
+      <c r="M23" s="2" t="n">
         <v>462.3585281434915</v>
       </c>
-      <c r="M23" s="2" t="n">
+      <c r="N23" s="2" t="n">
         <v>476.0153347549245</v>
       </c>
     </row>
@@ -1407,37 +1435,38 @@
           <t>Критическая скорость потока на выходе из ступени</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C24" s="1" t="inlineStr"/>
+      <c r="D24" s="2" t="n">
         <v>324.0777372086121</v>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="E24" s="2" t="n">
         <v>344.2854048832162</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="F24" s="2" t="n">
         <v>363.3124869844129</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="G24" s="2" t="n">
         <v>381.2871709710695</v>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>398.3196353879731</v>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="I24" s="2" t="n">
         <v>414.5573247272538</v>
       </c>
-      <c r="I24" s="2" t="n">
+      <c r="J24" s="2" t="n">
         <v>430.1468909948723</v>
       </c>
-      <c r="J24" s="2" t="n">
+      <c r="K24" s="2" t="n">
         <v>445.1457480100918</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="L24" s="2" t="n">
         <v>459.5750811212067</v>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="M24" s="2" t="n">
         <v>473.4519105373238</v>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="N24" s="2" t="n">
         <v>486.829421102413</v>
       </c>
     </row>
@@ -1452,37 +1481,38 @@
           <t>Относительный средний радиус на входе в ступень</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n">
+      <c r="C25" s="1" t="inlineStr"/>
+      <c r="D25" s="2" t="n">
         <v>0.7697077367416805</v>
       </c>
-      <c r="D25" s="2" t="n">
+      <c r="E25" s="2" t="n">
         <v>0.7842865295989352</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="F25" s="2" t="n">
         <v>0.8001506353803143</v>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="G25" s="2" t="n">
         <v>0.8172252054161926</v>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="H25" s="2" t="n">
         <v>0.8354360249081875</v>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="I25" s="2" t="n">
         <v>0.8547104687203072</v>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="J25" s="2" t="n">
         <v>0.874978249583736</v>
       </c>
-      <c r="J25" s="2" t="n">
+      <c r="K25" s="2" t="n">
         <v>0.8961719742482401</v>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="L25" s="2" t="n">
         <v>0.9182275294774144</v>
       </c>
-      <c r="L25" s="2" t="n">
+      <c r="M25" s="2" t="n">
         <v>0.9410843228060074</v>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="N25" s="2" t="n">
         <v>0.964685403461214</v>
       </c>
     </row>
@@ -1497,37 +1527,38 @@
           <t>Безразмерная окружная составляющая скорости на входе</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C26" s="1" t="inlineStr"/>
+      <c r="D26" s="2" t="n">
         <v>0.2209646382902902</v>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="E26" s="2" t="n">
         <v>0.2221096430231778</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="F26" s="2" t="n">
         <v>0.2247165257606272</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>0.228735252285246</v>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>0.2341340540041859</v>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="I26" s="2" t="n">
         <v>0.2408842262649444</v>
       </c>
-      <c r="I26" s="2" t="n">
+      <c r="J26" s="2" t="n">
         <v>0.2489829529108338</v>
       </c>
-      <c r="J26" s="2" t="n">
+      <c r="K26" s="2" t="n">
         <v>0.258436941975602</v>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="L26" s="2" t="n">
         <v>0.2692656201432488</v>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="M26" s="2" t="n">
         <v>0.2815002132115903</v>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="N26" s="2" t="n">
         <v>0.2951827699082133</v>
       </c>
     </row>
@@ -1542,37 +1573,38 @@
           <t>Угол абсолютной скорости на входе в РК</t>
         </is>
       </c>
-      <c r="C27" s="2" t="n">
+      <c r="C27" s="1" t="inlineStr"/>
+      <c r="D27" s="2" t="n">
         <v>1.194971328079617</v>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="E27" s="2" t="n">
         <v>1.180574579602314</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="F27" s="2" t="n">
         <v>1.162887574917572</v>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="G27" s="2" t="n">
         <v>1.141747321381765</v>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>1.116973003860716</v>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="I27" s="2" t="n">
         <v>1.088399301490598</v>
       </c>
-      <c r="I27" s="2" t="n">
+      <c r="J27" s="2" t="n">
         <v>1.05585028991713</v>
       </c>
-      <c r="J27" s="2" t="n">
+      <c r="K27" s="2" t="n">
         <v>1.019183822447235</v>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="L27" s="2" t="n">
         <v>0.9783090134087981</v>
       </c>
-      <c r="L27" s="2" t="n">
+      <c r="M27" s="2" t="n">
         <v>0.9332157000484604</v>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="N27" s="2" t="n">
         <v>0.8840072960802917</v>
       </c>
     </row>
@@ -1587,37 +1619,38 @@
           <t>Осевая скорость на входе в ступень</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C28" s="1" t="inlineStr"/>
+      <c r="D28" s="2" t="n">
         <v>179.267032761773</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="E28" s="2" t="n">
         <v>172.8646387345668</v>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="F28" s="2" t="n">
         <v>166.4622447073606</v>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>160.0598506801545</v>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>153.6574566529483</v>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="I28" s="2" t="n">
         <v>147.2550626257421</v>
       </c>
-      <c r="I28" s="2" t="n">
+      <c r="J28" s="2" t="n">
         <v>140.8526685985359</v>
       </c>
-      <c r="J28" s="2" t="n">
+      <c r="K28" s="2" t="n">
         <v>134.4502745713297</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="L28" s="2" t="n">
         <v>128.0478805441236</v>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="M28" s="2" t="n">
         <v>121.6454865169174</v>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="N28" s="2" t="n">
         <v>115.2430924897112</v>
       </c>
     </row>
@@ -1632,37 +1665,38 @@
           <t>Приведенная скорость на входе в ступень</t>
         </is>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C29" s="1" t="inlineStr"/>
+      <c r="D29" s="2" t="n">
         <v>0.6201721739235834</v>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="E29" s="2" t="n">
         <v>0.5642480089067109</v>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="F29" s="2" t="n">
         <v>0.5173169382832808</v>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>0.4772577835273439</v>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="H29" s="2" t="n">
         <v>0.4427623742092848</v>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="I29" s="2" t="n">
         <v>0.412838297016845</v>
       </c>
-      <c r="I29" s="2" t="n">
+      <c r="J29" s="2" t="n">
         <v>0.3867548721121836</v>
       </c>
-      <c r="J29" s="2" t="n">
+      <c r="K29" s="2" t="n">
         <v>0.3640913140459806</v>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="L29" s="2" t="n">
         <v>0.3443707830466253</v>
       </c>
-      <c r="L29" s="2" t="n">
+      <c r="M29" s="2" t="n">
         <v>0.3274240480592623</v>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="N29" s="2" t="n">
         <v>0.3130789351689683</v>
       </c>
     </row>
@@ -1677,37 +1711,38 @@
           <t>Газодинамическая функция расхода на входе</t>
         </is>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C30" s="1" t="inlineStr"/>
+      <c r="D30" s="2" t="n">
         <v>0.8289672515344797</v>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="E30" s="2" t="n">
         <v>0.7767379725045614</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="F30" s="2" t="n">
         <v>0.7282607559287695</v>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>0.6837140922479602</v>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="H30" s="2" t="n">
         <v>0.6432028517842318</v>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="I30" s="2" t="n">
         <v>0.6065518558070965</v>
       </c>
-      <c r="I30" s="2" t="n">
+      <c r="J30" s="2" t="n">
         <v>0.5735101964321142</v>
       </c>
-      <c r="J30" s="2" t="n">
+      <c r="K30" s="2" t="n">
         <v>0.5440703958039792</v>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="L30" s="2" t="n">
         <v>0.5178567173824349</v>
       </c>
-      <c r="L30" s="2" t="n">
+      <c r="M30" s="2" t="n">
         <v>0.4949503270135798</v>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="N30" s="2" t="n">
         <v>0.4753068980390184</v>
       </c>
     </row>
@@ -1722,37 +1757,38 @@
           <t>Кольцевая площадь на входе в ступень</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="C31" s="1" t="inlineStr"/>
+      <c r="D31" s="2" t="n">
         <v>0.3197918796405437</v>
       </c>
-      <c r="D31" s="2" t="n">
+      <c r="E31" s="2" t="n">
         <v>0.1333845085186511</v>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="F31" s="2" t="n">
         <v>0.09276327801446825</v>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>0.07559418092766981</v>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="H31" s="2" t="n">
         <v>0.06653889432920902</v>
       </c>
-      <c r="H31" s="2" t="n">
+      <c r="I31" s="2" t="n">
         <v>0.06128783511166349</v>
       </c>
-      <c r="I31" s="2" t="n">
+      <c r="J31" s="2" t="n">
         <v>0.05817197964158876</v>
       </c>
-      <c r="J31" s="2" t="n">
+      <c r="K31" s="2" t="n">
         <v>0.0563965166615289</v>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="L31" s="2" t="n">
         <v>0.05558444893690993</v>
       </c>
-      <c r="L31" s="2" t="n">
+      <c r="M31" s="2" t="n">
         <v>0.05549855900424231</v>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="N31" s="2" t="n">
         <v>0.0560173881283241</v>
       </c>
     </row>
@@ -1767,37 +1803,38 @@
           <t>Коэффициент расхода на выходе из ступени</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C32" s="1" t="inlineStr"/>
+      <c r="D32" s="2" t="n">
         <v>0.54</v>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="E32" s="2" t="n">
         <v>0.52</v>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="F32" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>0.48</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="H32" s="2" t="n">
         <v>0.46</v>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="I32" s="2" t="n">
         <v>0.44</v>
       </c>
-      <c r="I32" s="2" t="n">
+      <c r="J32" s="2" t="n">
         <v>0.42</v>
       </c>
-      <c r="J32" s="2" t="n">
+      <c r="K32" s="2" t="n">
         <v>0.4</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="L32" s="2" t="n">
         <v>0.38</v>
       </c>
-      <c r="L32" s="2" t="n">
+      <c r="M32" s="2" t="n">
         <v>0.36</v>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="N32" s="2" t="n">
         <v>0.34</v>
       </c>
     </row>
@@ -1812,37 +1849,38 @@
           <t>Осевая скорость на выходе из ступени</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n">
+      <c r="C33" s="1" t="inlineStr"/>
+      <c r="D33" s="2" t="n">
         <v>172.8646387345668</v>
       </c>
-      <c r="D33" s="2" t="n">
+      <c r="E33" s="2" t="n">
         <v>166.4622447073606</v>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="F33" s="2" t="n">
         <v>160.0598506801545</v>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>153.6574566529483</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="H33" s="2" t="n">
         <v>147.2550626257421</v>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="I33" s="2" t="n">
         <v>140.8526685985359</v>
       </c>
-      <c r="I33" s="2" t="n">
+      <c r="J33" s="2" t="n">
         <v>134.4502745713297</v>
       </c>
-      <c r="J33" s="2" t="n">
+      <c r="K33" s="2" t="n">
         <v>128.0478805441236</v>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="L33" s="2" t="n">
         <v>121.6454865169174</v>
       </c>
-      <c r="L33" s="2" t="n">
+      <c r="M33" s="2" t="n">
         <v>115.2430924897112</v>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="N33" s="2" t="n">
         <v>108.840698462505</v>
       </c>
     </row>
@@ -1857,37 +1895,38 @@
           <t>Приведенная скорость на выходе (1-е приближение)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C34" s="1" t="inlineStr"/>
+      <c r="D34" s="2" t="n">
         <v>0.5734271272297068</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="E34" s="2" t="n">
         <v>0.5228025526613771</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="F34" s="2" t="n">
         <v>0.4799344415446148</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>0.4431642821552224</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="H34" s="2" t="n">
         <v>0.4113261510914091</v>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="I34" s="2" t="n">
         <v>0.3835331465108897</v>
       </c>
-      <c r="I34" s="2" t="n">
+      <c r="J34" s="2" t="n">
         <v>0.3591420777761956</v>
       </c>
-      <c r="J34" s="2" t="n">
+      <c r="K34" s="2" t="n">
         <v>0.3377484939263771</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="L34" s="2" t="n">
         <v>0.3190764313863512</v>
       </c>
-      <c r="L34" s="2" t="n">
+      <c r="M34" s="2" t="n">
         <v>0.3029231587547552</v>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="N34" s="2" t="n">
         <v>0.2891175076909822</v>
       </c>
     </row>
@@ -1902,37 +1941,38 @@
           <t>Газодинамическая функция расхода на выходе</t>
         </is>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C35" s="1" t="inlineStr"/>
+      <c r="D35" s="2" t="n">
         <v>0.785749222309033</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="E35" s="2" t="n">
         <v>0.7341503741161742</v>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="F35" s="2" t="n">
         <v>0.6867841552835888</v>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>0.6436876257254293</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="H35" s="2" t="n">
         <v>0.6046548160285634</v>
       </c>
-      <c r="H35" s="2" t="n">
+      <c r="I35" s="2" t="n">
         <v>0.5693399760999998</v>
       </c>
-      <c r="I35" s="2" t="n">
+      <c r="J35" s="2" t="n">
         <v>0.5375004202953272</v>
       </c>
-      <c r="J35" s="2" t="n">
+      <c r="K35" s="2" t="n">
         <v>0.5088838758809117</v>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="L35" s="2" t="n">
         <v>0.4834497779504509</v>
       </c>
-      <c r="L35" s="2" t="n">
+      <c r="M35" s="2" t="n">
         <v>0.461124988676336</v>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="N35" s="2" t="n">
         <v>0.4418193991278718</v>
       </c>
     </row>
@@ -1947,37 +1987,38 @@
           <t>Кольцевая площадь на выходе (1-е приближение)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C36" s="1" t="inlineStr"/>
+      <c r="D36" s="2" t="n">
         <v>0.2715199844363019</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="E36" s="2" t="n">
         <v>0.1152518761147269</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="F36" s="2" t="n">
         <v>0.08133600902592081</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>0.06712407994818359</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="H36" s="2" t="n">
         <v>0.05975887380926437</v>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="I36" s="2" t="n">
         <v>0.05563589467254893</v>
       </c>
-      <c r="I36" s="2" t="n">
+      <c r="J36" s="2" t="n">
         <v>0.05327262404049409</v>
       </c>
-      <c r="J36" s="2" t="n">
+      <c r="K36" s="2" t="n">
         <v>0.05212041592284061</v>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="L36" s="2" t="n">
         <v>0.05184303068786426</v>
       </c>
-      <c r="L36" s="2" t="n">
+      <c r="M36" s="2" t="n">
         <v>0.05225713605927209</v>
       </c>
-      <c r="M36" s="2" t="n">
+      <c r="N36" s="2" t="n">
         <v>0.05327648247001738</v>
       </c>
     </row>
@@ -1992,37 +2033,38 @@
           <t>Относительный диаметр втулки на выходе (1-е приближение)</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n">
+      <c r="C37" s="1" t="inlineStr"/>
+      <c r="D37" s="2" t="n">
         <v>0.5621035277056677</v>
       </c>
-      <c r="D37" s="2" t="n">
+      <c r="E37" s="2" t="n">
         <v>0.8424050296758627</v>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="F37" s="2" t="n">
         <v>0.8916784139804044</v>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>0.9115341308345269</v>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="H37" s="2" t="n">
         <v>0.9216559104437274</v>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="I37" s="2" t="n">
         <v>0.9272737612921701</v>
       </c>
-      <c r="I37" s="2" t="n">
+      <c r="J37" s="2" t="n">
         <v>0.9304785920318749</v>
       </c>
-      <c r="J37" s="2" t="n">
+      <c r="K37" s="2" t="n">
         <v>0.9320371051015103</v>
       </c>
-      <c r="K37" s="2" t="n">
+      <c r="L37" s="2" t="n">
         <v>0.9324119160656946</v>
       </c>
-      <c r="L37" s="2" t="n">
+      <c r="M37" s="2" t="n">
         <v>0.9318523094273016</v>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="N37" s="2" t="n">
         <v>0.9304733686128156</v>
       </c>
     </row>
@@ -2037,37 +2079,38 @@
           <t>Относительный средний радиус на выходе из ступени</t>
         </is>
       </c>
-      <c r="C38" s="2" t="n">
+      <c r="C38" s="1" t="inlineStr"/>
+      <c r="D38" s="2" t="n">
         <v>0.8147901831335521</v>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="E38" s="2" t="n">
         <v>0.9291062724438937</v>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="F38" s="2" t="n">
         <v>0.9510901796604888</v>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>0.9600155362539734</v>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="H38" s="2" t="n">
         <v>0.9645299711897813</v>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="I38" s="2" t="n">
         <v>0.9669647075918497</v>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="J38" s="2" t="n">
         <v>0.9682510994927808</v>
       </c>
-      <c r="J38" s="2" t="n">
+      <c r="K38" s="2" t="n">
         <v>0.9687210437647382</v>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="L38" s="2" t="n">
         <v>0.9685643397409724</v>
       </c>
-      <c r="L38" s="2" t="n">
+      <c r="M38" s="2" t="n">
         <v>0.9678691439543144</v>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="N38" s="2" t="n">
         <v>0.9666562531855225</v>
       </c>
     </row>
@@ -2082,37 +2125,38 @@
           <t>Безразмерная окружная составляющая скорости на выходе</t>
         </is>
       </c>
-      <c r="C39" s="2" t="n">
+      <c r="C39" s="1" t="inlineStr"/>
+      <c r="D39" s="2" t="n">
         <v>0.2500657585861941</v>
       </c>
-      <c r="D39" s="2" t="n">
+      <c r="E39" s="2" t="n">
         <v>0.3180479671978335</v>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="F39" s="2" t="n">
         <v>0.3255888272795245</v>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>0.3247559975674831</v>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="H39" s="2" t="n">
         <v>0.3213200463991865</v>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="I39" s="2" t="n">
         <v>0.3168860663128854</v>
       </c>
-      <c r="I39" s="2" t="n">
+      <c r="J39" s="2" t="n">
         <v>0.3121645376277475</v>
       </c>
-      <c r="J39" s="2" t="n">
+      <c r="K39" s="2" t="n">
         <v>0.3074800309669942</v>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="L39" s="2" t="n">
         <v>0.3030876935226646</v>
       </c>
-      <c r="L39" s="2" t="n">
+      <c r="M39" s="2" t="n">
         <v>0.2991978289183804</v>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="N39" s="2" t="n">
         <v>0.295999401331859</v>
       </c>
     </row>
@@ -2127,37 +2171,38 @@
           <t>Угол абсолютной скорости на выходе из ступени</t>
         </is>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C40" s="1" t="inlineStr"/>
+      <c r="D40" s="2" t="n">
         <v>1.137114566119295</v>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="E40" s="2" t="n">
         <v>1.021868699911092</v>
       </c>
-      <c r="E40" s="2" t="n">
+      <c r="F40" s="2" t="n">
         <v>0.9935936749826273</v>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>0.9759654442114984</v>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="H40" s="2" t="n">
         <v>0.9610631051701353</v>
       </c>
-      <c r="H40" s="2" t="n">
+      <c r="I40" s="2" t="n">
         <v>0.9466444624942251</v>
       </c>
-      <c r="I40" s="2" t="n">
+      <c r="J40" s="2" t="n">
         <v>0.9316299423043648</v>
       </c>
-      <c r="J40" s="2" t="n">
+      <c r="K40" s="2" t="n">
         <v>0.9154341946829463</v>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="L40" s="2" t="n">
         <v>0.8975210063638877</v>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="M40" s="2" t="n">
         <v>0.8773745270752461</v>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="N40" s="2" t="n">
         <v>0.8544714971920427</v>
       </c>
     </row>
@@ -2172,37 +2217,38 @@
           <t>Приведенная скорость на выходе из ступени</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n">
+      <c r="C41" s="1" t="inlineStr"/>
+      <c r="D41" s="2" t="n">
         <v>0.5878226727702892</v>
       </c>
-      <c r="D41" s="2" t="n">
+      <c r="E41" s="2" t="n">
         <v>0.5667676571629278</v>
       </c>
-      <c r="E41" s="2" t="n">
+      <c r="F41" s="2" t="n">
         <v>0.5257290901455642</v>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>0.4865679818699653</v>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="H41" s="2" t="n">
         <v>0.4509518490978591</v>
       </c>
-      <c r="H41" s="2" t="n">
+      <c r="I41" s="2" t="n">
         <v>0.418710515432304</v>
       </c>
-      <c r="I41" s="2" t="n">
+      <c r="J41" s="2" t="n">
         <v>0.3894479028740119</v>
       </c>
-      <c r="J41" s="2" t="n">
+      <c r="K41" s="2" t="n">
         <v>0.3628203014767546</v>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="L41" s="2" t="n">
         <v>0.3385735337714739</v>
       </c>
-      <c r="L41" s="2" t="n">
+      <c r="M41" s="2" t="n">
         <v>0.3165023114321974</v>
       </c>
-      <c r="M41" s="2" t="n">
+      <c r="N41" s="2" t="n">
         <v>0.296424541748485</v>
       </c>
     </row>
@@ -2217,37 +2263,38 @@
           <t>Действительная кольцевая площадь на выходе из ступени</t>
         </is>
       </c>
-      <c r="C42" s="2" t="n">
+      <c r="C42" s="1" t="inlineStr"/>
+      <c r="D42" s="2" t="n">
         <v>0.2668338728927827</v>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="E42" s="2" t="n">
         <v>0.1085711657918483</v>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="F42" s="2" t="n">
         <v>0.07575720556651902</v>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>0.06221589109372239</v>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="H42" s="2" t="n">
         <v>0.0553185434035527</v>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="I42" s="2" t="n">
         <v>0.051585216662628</v>
       </c>
-      <c r="I42" s="2" t="n">
+      <c r="J42" s="2" t="n">
         <v>0.04960891500043527</v>
       </c>
-      <c r="J42" s="2" t="n">
+      <c r="K42" s="2" t="n">
         <v>0.04888627787204473</v>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="L42" s="2" t="n">
         <v>0.0491272818916562</v>
       </c>
-      <c r="L42" s="2" t="n">
+      <c r="M42" s="2" t="n">
         <v>0.05019599282151199</v>
       </c>
-      <c r="M42" s="2" t="n">
+      <c r="N42" s="2" t="n">
         <v>0.0520587088962016</v>
       </c>
     </row>
@@ -2262,37 +2309,38 @@
           <t>Кольцевая площадь на входе в следующую ступень</t>
         </is>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C43" s="1" t="inlineStr"/>
+      <c r="D43" s="2" t="n">
         <v>0.1085711657918483</v>
       </c>
-      <c r="D43" s="2" t="n">
+      <c r="E43" s="2" t="n">
         <v>0.07575720556651902</v>
       </c>
-      <c r="E43" s="2" t="n">
+      <c r="F43" s="2" t="n">
         <v>0.06221589109372239</v>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>0.0553185434035527</v>
       </c>
-      <c r="G43" s="2" t="n">
+      <c r="H43" s="2" t="n">
         <v>0.051585216662628</v>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="I43" s="2" t="n">
         <v>0.04960891500043527</v>
       </c>
-      <c r="I43" s="2" t="n">
+      <c r="J43" s="2" t="n">
         <v>0.04888627787204473</v>
       </c>
-      <c r="J43" s="2" t="n">
+      <c r="K43" s="2" t="n">
         <v>0.0491272818916562</v>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="L43" s="2" t="n">
         <v>0.05019599282151199</v>
       </c>
-      <c r="L43" s="2" t="n">
+      <c r="M43" s="2" t="n">
         <v>0.0520587088962016</v>
       </c>
-      <c r="M43" s="2" t="n">
+      <c r="N43" s="2" t="n">
         <v>0.05392142497089122</v>
       </c>
     </row>
@@ -2307,37 +2355,38 @@
           <t>Относительный диаметр втулки на выходе из ступени</t>
         </is>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C44" s="1" t="inlineStr"/>
+      <c r="D44" s="2" t="n">
         <v>0.5725085895090262</v>
       </c>
-      <c r="D44" s="2" t="n">
+      <c r="E44" s="2" t="n">
         <v>0.8523361607893765</v>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="F44" s="2" t="n">
         <v>0.8995249077670068</v>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>0.9182917073011213</v>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="H44" s="2" t="n">
         <v>0.9277047648075981</v>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="I44" s="2" t="n">
         <v>0.9327601467989414</v>
       </c>
-      <c r="I44" s="2" t="n">
+      <c r="J44" s="2" t="n">
         <v>0.9354252419824672</v>
       </c>
-      <c r="J44" s="2" t="n">
+      <c r="K44" s="2" t="n">
         <v>0.9363978434753509</v>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="L44" s="2" t="n">
         <v>0.9360735870836928</v>
       </c>
-      <c r="L44" s="2" t="n">
+      <c r="M44" s="2" t="n">
         <v>0.9346343454194882</v>
       </c>
-      <c r="M44" s="2" t="n">
+      <c r="N44" s="2" t="n">
         <v>0.9321204984578688</v>
       </c>
     </row>
@@ -2352,37 +2401,38 @@
           <t>Относительный средний радиус на выходе из РК</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C45" s="1" t="inlineStr"/>
+      <c r="D45" s="2" t="n">
         <v>0.7922489599376163</v>
       </c>
-      <c r="D45" s="2" t="n">
+      <c r="E45" s="2" t="n">
         <v>0.8566964010214144</v>
       </c>
-      <c r="E45" s="2" t="n">
+      <c r="F45" s="2" t="n">
         <v>0.8756204075204015</v>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>0.8886203708350831</v>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="H45" s="2" t="n">
         <v>0.8999829980489844</v>
       </c>
-      <c r="H45" s="2" t="n">
+      <c r="I45" s="2" t="n">
         <v>0.9108375881560784</v>
       </c>
-      <c r="I45" s="2" t="n">
+      <c r="J45" s="2" t="n">
         <v>0.9216146745382584</v>
       </c>
-      <c r="J45" s="2" t="n">
+      <c r="K45" s="2" t="n">
         <v>0.9324465090064892</v>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="L45" s="2" t="n">
         <v>0.9433959346091934</v>
       </c>
-      <c r="L45" s="2" t="n">
+      <c r="M45" s="2" t="n">
         <v>0.9544767333801609</v>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="N45" s="2" t="n">
         <v>0.9656708283233683</v>
       </c>
     </row>
@@ -2397,37 +2447,38 @@
           <t>Безразмерная окружная составляющая скорости на выходе из РК</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
+      <c r="C46" s="1" t="inlineStr"/>
+      <c r="D46" s="2" t="n">
         <v>0.5331301519094394</v>
       </c>
-      <c r="D46" s="2" t="n">
+      <c r="E46" s="2" t="n">
         <v>0.5146604548210467</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="F46" s="2" t="n">
         <v>0.5258374113682019</v>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>0.5412084154461251</v>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="H46" s="2" t="n">
         <v>0.5581764649226804</v>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="I46" s="2" t="n">
         <v>0.5760013884187075</v>
       </c>
-      <c r="I46" s="2" t="n">
+      <c r="J46" s="2" t="n">
         <v>0.5943180854893927</v>
       </c>
-      <c r="J46" s="2" t="n">
+      <c r="K46" s="2" t="n">
         <v>0.6129255216237373</v>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="L46" s="2" t="n">
         <v>0.6316485675547341</v>
       </c>
-      <c r="L46" s="2" t="n">
+      <c r="M46" s="2" t="n">
         <v>0.6503293830044945</v>
       </c>
-      <c r="M46" s="2" t="n">
+      <c r="N46" s="2" t="n">
         <v>0.6688194353854364</v>
       </c>
     </row>
@@ -2442,37 +2493,38 @@
           <t>Угол относительной скорости на входе в РК</t>
         </is>
       </c>
-      <c r="C47" s="2" t="n">
+      <c r="C47" s="1" t="inlineStr"/>
+      <c r="D47" s="2" t="n">
         <v>0.7955506638277184</v>
       </c>
-      <c r="D47" s="2" t="n">
+      <c r="E47" s="2" t="n">
         <v>0.7652798913021186</v>
       </c>
-      <c r="E47" s="2" t="n">
+      <c r="F47" s="2" t="n">
         <v>0.7348365983521747</v>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>0.7042804852547354</v>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="H47" s="2" t="n">
         <v>0.673683828398578</v>
       </c>
-      <c r="H47" s="2" t="n">
+      <c r="I47" s="2" t="n">
         <v>0.6431155521545162</v>
       </c>
-      <c r="I47" s="2" t="n">
+      <c r="J47" s="2" t="n">
         <v>0.6126566915509795</v>
       </c>
-      <c r="J47" s="2" t="n">
+      <c r="K47" s="2" t="n">
         <v>0.5823837334686925</v>
       </c>
-      <c r="K47" s="2" t="n">
+      <c r="L47" s="2" t="n">
         <v>0.5523686610810169</v>
       </c>
-      <c r="L47" s="2" t="n">
+      <c r="M47" s="2" t="n">
         <v>0.522676040644107</v>
       </c>
-      <c r="M47" s="2" t="n">
+      <c r="N47" s="2" t="n">
         <v>0.493360586253362</v>
       </c>
     </row>
@@ -2487,37 +2539,38 @@
           <t>Относительная осевая скорость на выходе из РК</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C48" s="1" t="inlineStr"/>
+      <c r="D48" s="2" t="n">
         <v>0.55</v>
       </c>
-      <c r="D48" s="2" t="n">
+      <c r="E48" s="2" t="n">
         <v>0.53</v>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="F48" s="2" t="n">
         <v>0.51</v>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>0.49</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="H48" s="2" t="n">
         <v>0.47</v>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="I48" s="2" t="n">
         <v>0.45</v>
       </c>
-      <c r="I48" s="2" t="n">
+      <c r="J48" s="2" t="n">
         <v>0.43</v>
       </c>
-      <c r="J48" s="2" t="n">
+      <c r="K48" s="2" t="n">
         <v>0.41</v>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="L48" s="2" t="n">
         <v>0.39</v>
       </c>
-      <c r="L48" s="2" t="n">
+      <c r="M48" s="2" t="n">
         <v>0.37</v>
       </c>
-      <c r="M48" s="2" t="n">
+      <c r="N48" s="2" t="n">
         <v>0.35</v>
       </c>
     </row>
@@ -2532,37 +2585,38 @@
           <t>Угол относительной скорости на выходе из РК</t>
         </is>
       </c>
-      <c r="C49" s="2" t="n">
+      <c r="C49" s="1" t="inlineStr"/>
+      <c r="D49" s="2" t="n">
         <v>1.130514300932322</v>
       </c>
-      <c r="D49" s="2" t="n">
+      <c r="E49" s="2" t="n">
         <v>0.9976963533957118</v>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="F49" s="2" t="n">
         <v>0.9696309402000549</v>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>0.9540529427009995</v>
       </c>
-      <c r="G49" s="2" t="n">
+      <c r="H49" s="2" t="n">
         <v>0.9420162509411002</v>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="I49" s="2" t="n">
         <v>0.9310945109634914</v>
       </c>
-      <c r="I49" s="2" t="n">
+      <c r="J49" s="2" t="n">
         <v>0.9201942496553147</v>
       </c>
-      <c r="J49" s="2" t="n">
+      <c r="K49" s="2" t="n">
         <v>0.9087932754368921</v>
       </c>
-      <c r="K49" s="2" t="n">
+      <c r="L49" s="2" t="n">
         <v>0.8964504952448477</v>
       </c>
-      <c r="L49" s="2" t="n">
+      <c r="M49" s="2" t="n">
         <v>0.8827721077517899</v>
       </c>
-      <c r="M49" s="2" t="n">
+      <c r="N49" s="2" t="n">
         <v>0.867379103508124</v>
       </c>
     </row>
@@ -2577,37 +2631,38 @@
           <t>Угол абсолютной скорости на выходе из РК</t>
         </is>
       </c>
-      <c r="C50" s="2" t="n">
+      <c r="C50" s="1" t="inlineStr"/>
+      <c r="D50" s="2" t="n">
         <v>0.8009719927700161</v>
       </c>
-      <c r="D50" s="2" t="n">
+      <c r="E50" s="2" t="n">
         <v>0.800080869900834</v>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="F50" s="2" t="n">
         <v>0.7701098785047441</v>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="G50" s="2" t="n">
         <v>0.7357802744699108</v>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="H50" s="2" t="n">
         <v>0.6998474394994911</v>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="I50" s="2" t="n">
         <v>0.6632018232964938</v>
       </c>
-      <c r="I50" s="2" t="n">
+      <c r="J50" s="2" t="n">
         <v>0.626336287717333</v>
       </c>
-      <c r="J50" s="2" t="n">
+      <c r="K50" s="2" t="n">
         <v>0.5895630781807731</v>
       </c>
-      <c r="K50" s="2" t="n">
+      <c r="L50" s="2" t="n">
         <v>0.5531385944983337</v>
       </c>
-      <c r="L50" s="2" t="n">
+      <c r="M50" s="2" t="n">
         <v>0.5172699628481386</v>
       </c>
-      <c r="M50" s="2" t="n">
+      <c r="N50" s="2" t="n">
         <v>0.4821213583193898</v>
       </c>
     </row>
@@ -2622,37 +2677,38 @@
           <t>Диффузность решетки РК</t>
         </is>
       </c>
-      <c r="C51" s="2" t="n">
+      <c r="C51" s="1" t="inlineStr"/>
+      <c r="D51" s="2" t="n">
         <v>0.3349636371046031</v>
       </c>
-      <c r="D51" s="2" t="n">
+      <c r="E51" s="2" t="n">
         <v>0.2324164620935932</v>
       </c>
-      <c r="E51" s="2" t="n">
+      <c r="F51" s="2" t="n">
         <v>0.2347943418478802</v>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="G51" s="2" t="n">
         <v>0.2497724574462641</v>
       </c>
-      <c r="G51" s="2" t="n">
+      <c r="H51" s="2" t="n">
         <v>0.2683324225425222</v>
       </c>
-      <c r="H51" s="2" t="n">
+      <c r="I51" s="2" t="n">
         <v>0.2879789588089752</v>
       </c>
-      <c r="I51" s="2" t="n">
+      <c r="J51" s="2" t="n">
         <v>0.3075375581043353</v>
       </c>
-      <c r="J51" s="2" t="n">
+      <c r="K51" s="2" t="n">
         <v>0.3264095419681996</v>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="L51" s="2" t="n">
         <v>0.3440818341638308</v>
       </c>
-      <c r="L51" s="2" t="n">
+      <c r="M51" s="2" t="n">
         <v>0.3600960671076829</v>
       </c>
-      <c r="M51" s="2" t="n">
+      <c r="N51" s="2" t="n">
         <v>0.374018517254762</v>
       </c>
     </row>
@@ -2667,37 +2723,38 @@
           <t>Диффузность решетки НА</t>
         </is>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C52" s="1" t="inlineStr"/>
+      <c r="D52" s="2" t="n">
         <v>0.3361425733492784</v>
       </c>
-      <c r="D52" s="2" t="n">
+      <c r="E52" s="2" t="n">
         <v>0.2217878300102584</v>
       </c>
-      <c r="E52" s="2" t="n">
+      <c r="F52" s="2" t="n">
         <v>0.2234837964778832</v>
       </c>
-      <c r="F52" s="2" t="n">
+      <c r="G52" s="2" t="n">
         <v>0.2401851697415877</v>
       </c>
-      <c r="G52" s="2" t="n">
+      <c r="H52" s="2" t="n">
         <v>0.2612156656706441</v>
       </c>
-      <c r="H52" s="2" t="n">
+      <c r="I52" s="2" t="n">
         <v>0.2834426391977313</v>
       </c>
-      <c r="I52" s="2" t="n">
+      <c r="J52" s="2" t="n">
         <v>0.3052936545870318</v>
       </c>
-      <c r="J52" s="2" t="n">
+      <c r="K52" s="2" t="n">
         <v>0.3258711165021732</v>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="L52" s="2" t="n">
         <v>0.344382411865554</v>
       </c>
-      <c r="L52" s="2" t="n">
+      <c r="M52" s="2" t="n">
         <v>0.3601045642271075</v>
       </c>
-      <c r="M52" s="2" t="n">
+      <c r="N52" s="2" t="n">
         <v>0.3723501388726529</v>
       </c>
     </row>
@@ -2712,37 +2769,38 @@
           <t>Относительная скорость на входе в РК</t>
         </is>
       </c>
-      <c r="C53" s="2" t="n">
+      <c r="C53" s="1" t="inlineStr"/>
+      <c r="D53" s="2" t="n">
         <v>250.9867050594529</v>
       </c>
-      <c r="D53" s="2" t="n">
+      <c r="E53" s="2" t="n">
         <v>249.5379481431306</v>
       </c>
-      <c r="E53" s="2" t="n">
+      <c r="F53" s="2" t="n">
         <v>248.2784541017162</v>
       </c>
-      <c r="F53" s="2" t="n">
+      <c r="G53" s="2" t="n">
         <v>247.2021510667909</v>
       </c>
-      <c r="G53" s="2" t="n">
+      <c r="H53" s="2" t="n">
         <v>246.2975394635712</v>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="I53" s="2" t="n">
         <v>245.551354564076</v>
       </c>
-      <c r="I53" s="2" t="n">
+      <c r="J53" s="2" t="n">
         <v>244.9428504897047</v>
       </c>
-      <c r="J53" s="2" t="n">
+      <c r="K53" s="2" t="n">
         <v>244.4478081615797</v>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="L53" s="2" t="n">
         <v>244.0378032431153</v>
       </c>
-      <c r="L53" s="2" t="n">
+      <c r="M53" s="2" t="n">
         <v>243.6805327507538</v>
       </c>
-      <c r="M53" s="2" t="n">
+      <c r="N53" s="2" t="n">
         <v>243.3402025335798</v>
       </c>
     </row>
@@ -2757,37 +2815,38 @@
           <t>Осевая скорость на выходе из РК</t>
         </is>
       </c>
-      <c r="C54" s="2" t="n">
+      <c r="C54" s="1" t="inlineStr"/>
+      <c r="D54" s="2" t="n">
         <v>176.0658357481699</v>
       </c>
-      <c r="D54" s="2" t="n">
+      <c r="E54" s="2" t="n">
         <v>169.6634417209637</v>
       </c>
-      <c r="E54" s="2" t="n">
+      <c r="F54" s="2" t="n">
         <v>163.2610476937575</v>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="G54" s="2" t="n">
         <v>156.8586536665514</v>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="H54" s="2" t="n">
         <v>150.4562596393452</v>
       </c>
-      <c r="H54" s="2" t="n">
+      <c r="I54" s="2" t="n">
         <v>144.053865612139</v>
       </c>
-      <c r="I54" s="2" t="n">
+      <c r="J54" s="2" t="n">
         <v>137.6514715849328</v>
       </c>
-      <c r="J54" s="2" t="n">
+      <c r="K54" s="2" t="n">
         <v>131.2490775577267</v>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="L54" s="2" t="n">
         <v>124.8466835305205</v>
       </c>
-      <c r="L54" s="2" t="n">
+      <c r="M54" s="2" t="n">
         <v>118.4442895033143</v>
       </c>
-      <c r="M54" s="2" t="n">
+      <c r="N54" s="2" t="n">
         <v>112.0418954761081</v>
       </c>
     </row>
@@ -2802,37 +2861,38 @@
           <t>Абсолютная скорость на выходе из РК</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
+      <c r="C55" s="1" t="inlineStr"/>
+      <c r="D55" s="2" t="n">
         <v>245.205790034887</v>
       </c>
-      <c r="D55" s="2" t="n">
+      <c r="E55" s="2" t="n">
         <v>236.4935905104464</v>
       </c>
-      <c r="E55" s="2" t="n">
+      <c r="F55" s="2" t="n">
         <v>234.498329779823</v>
       </c>
-      <c r="F55" s="2" t="n">
+      <c r="G55" s="2" t="n">
         <v>233.7107427554956</v>
       </c>
-      <c r="G55" s="2" t="n">
+      <c r="H55" s="2" t="n">
         <v>233.5910995314393</v>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="I55" s="2" t="n">
         <v>233.9892395892691</v>
       </c>
-      <c r="I55" s="2" t="n">
+      <c r="J55" s="2" t="n">
         <v>234.8278183206815</v>
       </c>
-      <c r="J55" s="2" t="n">
+      <c r="K55" s="2" t="n">
         <v>236.0603777859788</v>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="L55" s="2" t="n">
         <v>237.6400820277972</v>
       </c>
-      <c r="L55" s="2" t="n">
+      <c r="M55" s="2" t="n">
         <v>239.518922866217</v>
       </c>
-      <c r="M55" s="2" t="n">
+      <c r="N55" s="2" t="n">
         <v>241.6467913137315</v>
       </c>
     </row>
@@ -2847,37 +2907,38 @@
           <t>Температурная функция на входе в РК</t>
         </is>
       </c>
-      <c r="C56" s="2" t="n">
+      <c r="C56" s="1" t="inlineStr"/>
+      <c r="D56" s="2" t="n">
         <v>0.9359051796510285</v>
       </c>
-      <c r="D56" s="2" t="n">
+      <c r="E56" s="2" t="n">
         <v>0.9471884974081952</v>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="F56" s="2" t="n">
         <v>0.9558468274253789</v>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="G56" s="2" t="n">
         <v>0.9625962844363063</v>
       </c>
-      <c r="G56" s="2" t="n">
+      <c r="H56" s="2" t="n">
         <v>0.9680176322189936</v>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="I56" s="2" t="n">
         <v>0.9724188180361157</v>
       </c>
-      <c r="I56" s="2" t="n">
+      <c r="J56" s="2" t="n">
         <v>0.9759918453834303</v>
       </c>
-      <c r="J56" s="2" t="n">
+      <c r="K56" s="2" t="n">
         <v>0.9789558341494647</v>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="L56" s="2" t="n">
         <v>0.9813382851974597</v>
       </c>
-      <c r="L56" s="2" t="n">
+      <c r="M56" s="2" t="n">
         <v>0.9832888381701964</v>
       </c>
-      <c r="M56" s="2" t="n">
+      <c r="N56" s="2" t="n">
         <v>0.9848744817582111</v>
       </c>
     </row>
@@ -2892,37 +2953,38 @@
           <t>Статическая температура на входе в РК</t>
         </is>
       </c>
-      <c r="C57" s="2" t="n">
+      <c r="C57" s="1" t="inlineStr"/>
+      <c r="D57" s="2" t="n">
         <v>269.5406917394962</v>
       </c>
-      <c r="D57" s="2" t="n">
+      <c r="E57" s="2" t="n">
         <v>310.2058455736416</v>
       </c>
-      <c r="E57" s="2" t="n">
+      <c r="F57" s="2" t="n">
         <v>350.7990404931795</v>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="G57" s="2" t="n">
         <v>391.300306340105</v>
       </c>
-      <c r="G57" s="2" t="n">
+      <c r="H57" s="2" t="n">
         <v>431.7424565133022</v>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="I57" s="2" t="n">
         <v>472.1176143031199</v>
       </c>
-      <c r="I57" s="2" t="n">
+      <c r="J57" s="2" t="n">
         <v>512.4056891025803</v>
       </c>
-      <c r="J57" s="2" t="n">
+      <c r="K57" s="2" t="n">
         <v>552.6322356915423</v>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="L57" s="2" t="n">
         <v>592.7416907832766</v>
       </c>
-      <c r="L57" s="2" t="n">
+      <c r="M57" s="2" t="n">
         <v>632.7614345909392</v>
       </c>
-      <c r="M57" s="2" t="n">
+      <c r="N57" s="2" t="n">
         <v>672.6860394027558</v>
       </c>
     </row>
@@ -2937,37 +2999,38 @@
           <t>Скорость звука на входе в РК</t>
         </is>
       </c>
-      <c r="C58" s="2" t="n">
+      <c r="C58" s="1" t="inlineStr"/>
+      <c r="D58" s="2" t="n">
         <v>300.6251763668889</v>
       </c>
-      <c r="D58" s="2" t="n">
+      <c r="E58" s="2" t="n">
         <v>322.3999014125897</v>
       </c>
-      <c r="E58" s="2" t="n">
+      <c r="F58" s="2" t="n">
         <v>342.7149378286148</v>
       </c>
-      <c r="F58" s="2" t="n">
+      <c r="G58" s="2" t="n">
         <v>361.8385052109181</v>
       </c>
-      <c r="G58" s="2" t="n">
+      <c r="H58" s="2" t="n">
         <v>379.9026907528486</v>
       </c>
-      <c r="H58" s="2" t="n">
+      <c r="I58" s="2" t="n">
         <v>397.0446523527072</v>
       </c>
-      <c r="I58" s="2" t="n">
+      <c r="J58" s="2" t="n">
         <v>413.4031356106535</v>
       </c>
-      <c r="J58" s="2" t="n">
+      <c r="K58" s="2" t="n">
         <v>428.9989021073237</v>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="L58" s="2" t="n">
         <v>444.0283162357795</v>
       </c>
-      <c r="L58" s="2" t="n">
+      <c r="M58" s="2" t="n">
         <v>458.4789778163817</v>
       </c>
-      <c r="M58" s="2" t="n">
+      <c r="N58" s="2" t="n">
         <v>472.401628579361</v>
       </c>
     </row>
@@ -2982,37 +3045,38 @@
           <t>Число Маха относительной скорости на входе в РК</t>
         </is>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C59" s="1" t="inlineStr"/>
+      <c r="D59" s="2" t="n">
         <v>0.8348825207944121</v>
       </c>
-      <c r="D59" s="2" t="n">
+      <c r="E59" s="2" t="n">
         <v>0.7740013165319974</v>
       </c>
-      <c r="E59" s="2" t="n">
+      <c r="F59" s="2" t="n">
         <v>0.7244459657194036</v>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="G59" s="2" t="n">
         <v>0.6831836510121971</v>
       </c>
-      <c r="G59" s="2" t="n">
+      <c r="H59" s="2" t="n">
         <v>0.6483174388038324</v>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="I59" s="2" t="n">
         <v>0.6184477063449908</v>
       </c>
-      <c r="I59" s="2" t="n">
+      <c r="J59" s="2" t="n">
         <v>0.5925036106170077</v>
       </c>
-      <c r="J59" s="2" t="n">
+      <c r="K59" s="2" t="n">
         <v>0.5698098688849922</v>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="L59" s="2" t="n">
         <v>0.5495996411038141</v>
       </c>
-      <c r="L59" s="2" t="n">
+      <c r="M59" s="2" t="n">
         <v>0.5314977229955928</v>
       </c>
-      <c r="M59" s="2" t="n">
+      <c r="N59" s="2" t="n">
         <v>0.515112962809568</v>
       </c>
     </row>
@@ -3027,37 +3091,38 @@
           <t>Приведенная абсолютная скорость на выходе из РК</t>
         </is>
       </c>
-      <c r="C60" s="2" t="n">
+      <c r="C60" s="1" t="inlineStr"/>
+      <c r="D60" s="2" t="n">
         <v>0.7566264568091747</v>
       </c>
-      <c r="D60" s="2" t="n">
+      <c r="E60" s="2" t="n">
         <v>0.6869114611194933</v>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="F60" s="2" t="n">
         <v>0.6454452796990806</v>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="G60" s="2" t="n">
         <v>0.6129520229077641</v>
       </c>
-      <c r="G60" s="2" t="n">
+      <c r="H60" s="2" t="n">
         <v>0.586441337002922</v>
       </c>
-      <c r="H60" s="2" t="n">
+      <c r="I60" s="2" t="n">
         <v>0.5644315650271423</v>
       </c>
-      <c r="I60" s="2" t="n">
+      <c r="J60" s="2" t="n">
         <v>0.5459247137124625</v>
       </c>
-      <c r="J60" s="2" t="n">
+      <c r="K60" s="2" t="n">
         <v>0.5302990735983107</v>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="L60" s="2" t="n">
         <v>0.5170865257707974</v>
       </c>
-      <c r="L60" s="2" t="n">
+      <c r="M60" s="2" t="n">
         <v>0.505899157940635</v>
       </c>
-      <c r="M60" s="2" t="n">
+      <c r="N60" s="2" t="n">
         <v>0.4963685037081949</v>
       </c>
     </row>
@@ -3072,37 +3137,38 @@
           <t>Полная температура на выходе из РК</t>
         </is>
       </c>
-      <c r="C61" s="2" t="n">
+      <c r="C61" s="1" t="inlineStr"/>
+      <c r="D61" s="2" t="n">
         <v>313.442997929923</v>
       </c>
-      <c r="D61" s="2" t="n">
+      <c r="E61" s="2" t="n">
         <v>354.0214305740254</v>
       </c>
-      <c r="E61" s="2" t="n">
+      <c r="F61" s="2" t="n">
         <v>394.4947937841117</v>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="G61" s="2" t="n">
         <v>434.8949904414187</v>
       </c>
-      <c r="G61" s="2" t="n">
+      <c r="H61" s="2" t="n">
         <v>475.1545947444316</v>
       </c>
-      <c r="H61" s="2" t="n">
+      <c r="I61" s="2" t="n">
         <v>515.2708761709553</v>
       </c>
-      <c r="I61" s="2" t="n">
+      <c r="J61" s="2" t="n">
         <v>555.5938493530826</v>
       </c>
-      <c r="J61" s="2" t="n">
+      <c r="K61" s="2" t="n">
         <v>595.7288057964814</v>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="L61" s="2" t="n">
         <v>635.7905853599461</v>
       </c>
-      <c r="L61" s="2" t="n">
+      <c r="M61" s="2" t="n">
         <v>675.6805057771428</v>
       </c>
-      <c r="M61" s="2" t="n">
+      <c r="N61" s="2" t="n">
         <v>715.3766483915773</v>
       </c>
     </row>
@@ -3117,37 +3183,38 @@
           <t>Температурная функция на выходе из РК</t>
         </is>
       </c>
-      <c r="C62" s="2" t="n">
+      <c r="C62" s="1" t="inlineStr"/>
+      <c r="D62" s="2" t="n">
         <v>0.9050376398220753</v>
       </c>
-      <c r="D62" s="2" t="n">
+      <c r="E62" s="2" t="n">
         <v>0.9221515369239762</v>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="F62" s="2" t="n">
         <v>0.9315887440071891</v>
       </c>
-      <c r="F62" s="2" t="n">
+      <c r="G62" s="2" t="n">
         <v>0.9387054073290569</v>
       </c>
-      <c r="G62" s="2" t="n">
+      <c r="H62" s="2" t="n">
         <v>0.9443452715453308</v>
       </c>
-      <c r="H62" s="2" t="n">
+      <c r="I62" s="2" t="n">
         <v>0.9488659986366965</v>
       </c>
-      <c r="I62" s="2" t="n">
+      <c r="J62" s="2" t="n">
         <v>0.9526874245639199</v>
       </c>
-      <c r="J62" s="2" t="n">
+      <c r="K62" s="2" t="n">
         <v>0.9557472067545164</v>
       </c>
-      <c r="K62" s="2" t="n">
+      <c r="L62" s="2" t="n">
         <v>0.9583215134744612</v>
       </c>
-      <c r="L62" s="2" t="n">
+      <c r="M62" s="2" t="n">
         <v>0.9605060583055894</v>
       </c>
-      <c r="M62" s="2" t="n">
+      <c r="N62" s="2" t="n">
         <v>0.9623671724133392</v>
       </c>
     </row>
@@ -3162,37 +3229,38 @@
           <t>Статическая температура на выходе из РК</t>
         </is>
       </c>
-      <c r="C63" s="2" t="n">
+      <c r="C63" s="1" t="inlineStr"/>
+      <c r="D63" s="2" t="n">
         <v>618.1561170673046</v>
       </c>
-      <c r="D63" s="2" t="n">
+      <c r="E63" s="2" t="n">
         <v>629.8452001671857</v>
       </c>
-      <c r="E63" s="2" t="n">
+      <c r="F63" s="2" t="n">
         <v>636.2909732818439</v>
       </c>
-      <c r="F63" s="2" t="n">
+      <c r="G63" s="2" t="n">
         <v>641.1517754981871</v>
       </c>
-      <c r="G63" s="2" t="n">
+      <c r="H63" s="2" t="n">
         <v>645.0038987815944</v>
       </c>
-      <c r="H63" s="2" t="n">
+      <c r="I63" s="2" t="n">
         <v>648.0916323543871</v>
       </c>
-      <c r="I63" s="2" t="n">
+      <c r="J63" s="2" t="n">
         <v>650.7017313258477</v>
       </c>
-      <c r="J63" s="2" t="n">
+      <c r="K63" s="2" t="n">
         <v>652.7916146575318</v>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="L63" s="2" t="n">
         <v>654.54990997711</v>
       </c>
-      <c r="L63" s="2" t="n">
+      <c r="M63" s="2" t="n">
         <v>656.0419912905846</v>
       </c>
-      <c r="M63" s="2" t="n">
+      <c r="N63" s="2" t="n">
         <v>657.3131639132968</v>
       </c>
     </row>
@@ -3207,37 +3275,38 @@
           <t>Скорость звука на выходе из РК</t>
         </is>
       </c>
-      <c r="C64" s="2" t="n">
+      <c r="C64" s="1" t="inlineStr"/>
+      <c r="D64" s="2" t="n">
         <v>455.1878653606111</v>
       </c>
-      <c r="D64" s="2" t="n">
+      <c r="E64" s="2" t="n">
         <v>459.3078267797998</v>
       </c>
-      <c r="E64" s="2" t="n">
+      <c r="F64" s="2" t="n">
         <v>461.4872296915951</v>
       </c>
-      <c r="F64" s="2" t="n">
+      <c r="G64" s="2" t="n">
         <v>463.0632867898798</v>
       </c>
-      <c r="G64" s="2" t="n">
+      <c r="H64" s="2" t="n">
         <v>464.2141998143966</v>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="I64" s="2" t="n">
         <v>465.0598657953267</v>
       </c>
-      <c r="I64" s="2" t="n">
+      <c r="J64" s="2" t="n">
         <v>465.6865011908989</v>
       </c>
-      <c r="J64" s="2" t="n">
+      <c r="K64" s="2" t="n">
         <v>466.1175242700996</v>
       </c>
-      <c r="K64" s="2" t="n">
+      <c r="L64" s="2" t="n">
         <v>466.4555110608122</v>
       </c>
-      <c r="L64" s="2" t="n">
+      <c r="M64" s="2" t="n">
         <v>466.6790527756584</v>
       </c>
-      <c r="M64" s="2" t="n">
+      <c r="N64" s="2" t="n">
         <v>466.8137721497224</v>
       </c>
     </row>
@@ -3252,37 +3321,38 @@
           <t>Среднее число Маха на выходе из РК</t>
         </is>
       </c>
-      <c r="C65" s="2" t="n">
+      <c r="C65" s="1" t="inlineStr"/>
+      <c r="D65" s="2" t="n">
         <v>0.5386914034727813</v>
       </c>
-      <c r="D65" s="2" t="n">
+      <c r="E65" s="2" t="n">
         <v>0.514891270563577</v>
       </c>
-      <c r="E65" s="2" t="n">
+      <c r="F65" s="2" t="n">
         <v>0.5081361188185742</v>
       </c>
-      <c r="F65" s="2" t="n">
+      <c r="G65" s="2" t="n">
         <v>0.5047058348668969</v>
       </c>
-      <c r="G65" s="2" t="n">
+      <c r="H65" s="2" t="n">
         <v>0.5031967992897124</v>
       </c>
-      <c r="H65" s="2" t="n">
+      <c r="I65" s="2" t="n">
         <v>0.5031378899770466</v>
       </c>
-      <c r="I65" s="2" t="n">
+      <c r="J65" s="2" t="n">
         <v>0.5042615959881958</v>
       </c>
-      <c r="J65" s="2" t="n">
+      <c r="K65" s="2" t="n">
         <v>0.5064396112453169</v>
       </c>
-      <c r="K65" s="2" t="n">
+      <c r="L65" s="2" t="n">
         <v>0.5094592654449651</v>
       </c>
-      <c r="L65" s="2" t="n">
+      <c r="M65" s="2" t="n">
         <v>0.5132412124384729</v>
       </c>
-      <c r="M65" s="2" t="n">
+      <c r="N65" s="2" t="n">
         <v>0.5176513756244266</v>
       </c>
     </row>

</xml_diff>